<commit_message>
Update all prices (col D) and discounts (col F) for all products including hardcoded HTML
</commit_message>
<xml_diff>
--- a/tabela_produtos_site.xlsx
+++ b/tabela_produtos_site.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0925d356f97d17c9/Desktop/special-summer-sale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="460" documentId="11_1479D0EED2335F840378C78657AD3C1B78FA1F78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE56C006-6895-4636-BA08-D53162748D67}"/>
+  <xr:revisionPtr revIDLastSave="521" documentId="11_1479D0EED2335F840378C78657AD3C1B78FA1F78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{488128B3-D6A2-4B33-AE83-900A21C6F11A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2162,6 +2161,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2267,13 +2269,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3966,9 +3968,7 @@
       <c r="D35" s="11">
         <v>1450</v>
       </c>
-      <c r="E35" s="1">
-        <v>870</v>
-      </c>
+      <c r="E35" s="1"/>
       <c r="F35" s="1">
         <v>0.3</v>
       </c>
@@ -4007,9 +4007,7 @@
       <c r="D36" s="11">
         <v>3614</v>
       </c>
-      <c r="E36" s="1">
-        <v>1445.6</v>
-      </c>
+      <c r="E36" s="1"/>
       <c r="F36" s="1">
         <v>0.6</v>
       </c>
@@ -4048,9 +4046,7 @@
       <c r="D37" s="11">
         <v>6624</v>
       </c>
-      <c r="E37" s="1">
-        <v>2649.6</v>
-      </c>
+      <c r="E37" s="1"/>
       <c r="F37" s="1">
         <v>0.6</v>
       </c>
@@ -4089,9 +4085,7 @@
       <c r="D38" s="11">
         <v>6350</v>
       </c>
-      <c r="E38" s="1">
-        <v>2540</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="1">
         <v>0.6</v>
       </c>
@@ -4130,9 +4124,7 @@
       <c r="D39" s="11">
         <v>3734</v>
       </c>
-      <c r="E39" s="1">
-        <v>1493.6</v>
-      </c>
+      <c r="E39" s="1"/>
       <c r="F39" s="1">
         <v>0.6</v>
       </c>
@@ -4171,9 +4163,7 @@
       <c r="D40" s="11">
         <v>2890</v>
       </c>
-      <c r="E40" s="1">
-        <v>1156</v>
-      </c>
+      <c r="E40" s="1"/>
       <c r="F40" s="1">
         <v>0.6</v>
       </c>
@@ -4212,9 +4202,7 @@
       <c r="D41" s="11">
         <v>3455</v>
       </c>
-      <c r="E41" s="1">
-        <v>1382</v>
-      </c>
+      <c r="E41" s="1"/>
       <c r="F41" s="1">
         <v>0.6</v>
       </c>
@@ -4253,9 +4241,7 @@
       <c r="D42" s="11">
         <v>8700</v>
       </c>
-      <c r="E42" s="1">
-        <v>3480</v>
-      </c>
+      <c r="E42" s="1"/>
       <c r="F42" s="1">
         <v>0.4</v>
       </c>
@@ -4294,9 +4280,7 @@
       <c r="D43" s="11">
         <v>4525</v>
       </c>
-      <c r="E43" s="1">
-        <v>2715</v>
-      </c>
+      <c r="E43" s="1"/>
       <c r="F43" s="1">
         <v>0.4</v>
       </c>
@@ -4335,9 +4319,7 @@
       <c r="D44" s="11">
         <v>2750</v>
       </c>
-      <c r="E44" s="1">
-        <v>1650</v>
-      </c>
+      <c r="E44" s="1"/>
       <c r="F44" s="1">
         <v>0.3</v>
       </c>
@@ -4378,9 +4360,7 @@
       <c r="D45" s="11">
         <v>1300</v>
       </c>
-      <c r="E45" s="1">
-        <v>909.99999999999989</v>
-      </c>
+      <c r="E45" s="1"/>
       <c r="F45" s="1">
         <v>0.2</v>
       </c>
@@ -4419,9 +4399,7 @@
       <c r="D46" s="11">
         <v>5880</v>
       </c>
-      <c r="E46" s="1">
-        <v>2640</v>
-      </c>
+      <c r="E46" s="1"/>
       <c r="F46" s="1">
         <v>0.5</v>
       </c>
@@ -4462,9 +4440,7 @@
       <c r="D47" s="11">
         <v>1455</v>
       </c>
-      <c r="E47" s="1">
-        <v>727.5</v>
-      </c>
+      <c r="E47" s="1"/>
       <c r="F47" s="1">
         <v>0.4</v>
       </c>
@@ -4501,9 +4477,7 @@
       <c r="D48" s="11">
         <v>3360</v>
       </c>
-      <c r="E48" s="1">
-        <v>2352</v>
-      </c>
+      <c r="E48" s="1"/>
       <c r="F48" s="1">
         <v>0.3</v>
       </c>
@@ -4542,11 +4516,9 @@
         <v>185</v>
       </c>
       <c r="D49" s="11">
-        <v>2600</v>
-      </c>
-      <c r="E49" s="1">
-        <v>1300</v>
-      </c>
+        <v>2980</v>
+      </c>
+      <c r="E49" s="1"/>
       <c r="F49" s="1">
         <v>0.5</v>
       </c>
@@ -4583,11 +4555,9 @@
         <v>188</v>
       </c>
       <c r="D50" s="11">
-        <v>2700</v>
-      </c>
-      <c r="E50" s="1">
-        <v>1350</v>
-      </c>
+        <v>2980</v>
+      </c>
+      <c r="E50" s="1"/>
       <c r="F50" s="1">
         <v>0.5</v>
       </c>
@@ -4626,9 +4596,7 @@
       <c r="D51" s="11">
         <v>1752</v>
       </c>
-      <c r="E51" s="1">
-        <v>700.80000000000007</v>
-      </c>
+      <c r="E51" s="1"/>
       <c r="F51" s="1">
         <v>0.4</v>
       </c>
@@ -4667,9 +4635,7 @@
       <c r="D52" s="11">
         <v>1590</v>
       </c>
-      <c r="E52" s="1">
-        <v>636</v>
-      </c>
+      <c r="E52" s="1"/>
       <c r="F52" s="1">
         <v>0.4</v>
       </c>
@@ -4708,9 +4674,7 @@
       <c r="D53" s="11">
         <v>1590</v>
       </c>
-      <c r="E53" s="1">
-        <v>954</v>
-      </c>
+      <c r="E53" s="1"/>
       <c r="F53" s="1">
         <v>0.3</v>
       </c>
@@ -4749,9 +4713,7 @@
       <c r="D54" s="11">
         <v>1590</v>
       </c>
-      <c r="E54" s="1">
-        <v>795</v>
-      </c>
+      <c r="E54" s="1"/>
       <c r="F54" s="1">
         <v>0.4</v>
       </c>
@@ -4790,9 +4752,7 @@
       <c r="D55" s="11">
         <v>1752</v>
       </c>
-      <c r="E55" s="1">
-        <v>1051.2</v>
-      </c>
+      <c r="E55" s="1"/>
       <c r="F55" s="1">
         <v>0.4</v>
       </c>
@@ -4831,9 +4791,7 @@
       <c r="D56" s="11">
         <v>1560</v>
       </c>
-      <c r="E56" s="1">
-        <v>780</v>
-      </c>
+      <c r="E56" s="1"/>
       <c r="F56" s="1">
         <v>0.4</v>
       </c>
@@ -4872,9 +4830,7 @@
       <c r="D57" s="11">
         <v>2980</v>
       </c>
-      <c r="E57" s="1">
-        <v>1192</v>
-      </c>
+      <c r="E57" s="1"/>
       <c r="F57" s="1">
         <v>0.5</v>
       </c>
@@ -4913,9 +4869,7 @@
       <c r="D58" s="11">
         <v>3745</v>
       </c>
-      <c r="E58" s="1">
-        <v>1872.5</v>
-      </c>
+      <c r="E58" s="1"/>
       <c r="F58" s="1">
         <v>0.5</v>
       </c>
@@ -4954,9 +4908,7 @@
       <c r="D59" s="11">
         <v>2980</v>
       </c>
-      <c r="E59" s="1">
-        <v>1490</v>
-      </c>
+      <c r="E59" s="1"/>
       <c r="F59" s="1">
         <v>0.5</v>
       </c>
@@ -4997,9 +4949,7 @@
       <c r="D60" s="11">
         <v>980</v>
       </c>
-      <c r="E60" s="1">
-        <v>588</v>
-      </c>
+      <c r="E60" s="1"/>
       <c r="F60" s="1">
         <v>0.4</v>
       </c>
@@ -5040,9 +4990,7 @@
       <c r="D61" s="11">
         <v>3700</v>
       </c>
-      <c r="E61" s="1">
-        <v>1850</v>
-      </c>
+      <c r="E61" s="1"/>
       <c r="F61" s="1">
         <v>0.5</v>
       </c>
@@ -5081,9 +5029,7 @@
       <c r="D62" s="11">
         <v>670</v>
       </c>
-      <c r="E62" s="1">
-        <v>468.99999999999989</v>
-      </c>
+      <c r="E62" s="1"/>
       <c r="F62" s="1">
         <v>0.3</v>
       </c>
@@ -5122,9 +5068,7 @@
       <c r="D63" s="11">
         <v>1803</v>
       </c>
-      <c r="E63" s="1">
-        <v>1262.0999999999999</v>
-      </c>
+      <c r="E63" s="1"/>
       <c r="F63" s="1">
         <v>0.2</v>
       </c>
@@ -5163,9 +5107,7 @@
       <c r="D64" s="11">
         <v>1595</v>
       </c>
-      <c r="E64" s="1">
-        <v>1116.5</v>
-      </c>
+      <c r="E64" s="1"/>
       <c r="F64" s="1">
         <v>0.2</v>
       </c>
@@ -5204,9 +5146,7 @@
       <c r="D65" s="11">
         <v>6070</v>
       </c>
-      <c r="E65" s="1">
-        <v>2428</v>
-      </c>
+      <c r="E65" s="1"/>
       <c r="F65" s="1">
         <v>0.6</v>
       </c>
@@ -5245,9 +5185,7 @@
       <c r="D66" s="11">
         <v>28588</v>
       </c>
-      <c r="E66" s="1">
-        <v>11435.2</v>
-      </c>
+      <c r="E66" s="1"/>
       <c r="F66" s="1">
         <v>0.5</v>
       </c>
@@ -5286,11 +5224,9 @@
       <c r="D67" s="11">
         <v>9674</v>
       </c>
-      <c r="E67" s="1">
-        <v>6771.7999999999993</v>
-      </c>
+      <c r="E67" s="1"/>
       <c r="F67" s="1">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" s="1" t="s">
@@ -5329,11 +5265,9 @@
       <c r="D68" s="11">
         <v>16358</v>
       </c>
-      <c r="E68" s="1">
-        <v>8179</v>
-      </c>
+      <c r="E68" s="1"/>
       <c r="F68" s="1">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" s="1" t="s">
@@ -5372,9 +5306,7 @@
       <c r="D69" s="11">
         <v>7570</v>
       </c>
-      <c r="E69" s="1">
-        <v>3028</v>
-      </c>
+      <c r="E69" s="1"/>
       <c r="F69" s="1">
         <v>0.5</v>
       </c>
@@ -6249,10 +6181,10 @@
       <c r="C91" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="D91" s="11"/>
-      <c r="E91" s="1">
-        <v>1992</v>
-      </c>
+      <c r="D91" s="11">
+        <v>4980</v>
+      </c>
+      <c r="E91" s="1"/>
       <c r="F91" s="1">
         <v>0.6</v>
       </c>
@@ -6288,10 +6220,10 @@
       <c r="C92" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="D92" s="11"/>
-      <c r="E92" s="1">
-        <v>864.5</v>
-      </c>
+      <c r="D92" s="11">
+        <v>1720</v>
+      </c>
+      <c r="E92" s="1"/>
       <c r="F92" s="1">
         <v>0.4</v>
       </c>
@@ -6327,12 +6259,12 @@
       <c r="C93" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="D93" s="11"/>
-      <c r="E93" s="1">
-        <v>717.5</v>
-      </c>
+      <c r="D93" s="11">
+        <v>1435</v>
+      </c>
+      <c r="E93" s="1"/>
       <c r="F93" s="1">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" s="1" t="s">
@@ -6366,10 +6298,10 @@
       <c r="C94" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="D94" s="11"/>
-      <c r="E94" s="1">
-        <v>2252.5</v>
-      </c>
+      <c r="D94" s="11">
+        <v>3980</v>
+      </c>
+      <c r="E94" s="1"/>
       <c r="F94" s="1">
         <v>0.5</v>
       </c>
@@ -6405,10 +6337,10 @@
       <c r="C95" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="D95" s="11"/>
-      <c r="E95" s="1">
-        <v>1475</v>
-      </c>
+      <c r="D95" s="11">
+        <v>2950</v>
+      </c>
+      <c r="E95" s="1"/>
       <c r="F95" s="1">
         <v>0.4</v>
       </c>
@@ -6444,10 +6376,10 @@
       <c r="C96" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="D96" s="11"/>
-      <c r="E96" s="1">
-        <v>2283.6</v>
-      </c>
+      <c r="D96" s="11">
+        <v>3806</v>
+      </c>
+      <c r="E96" s="1"/>
       <c r="F96" s="1">
         <v>0.4</v>
       </c>
@@ -6483,12 +6415,12 @@
       <c r="C97" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="D97" s="11"/>
-      <c r="E97" s="1">
-        <v>820</v>
-      </c>
+      <c r="D97" s="11">
+        <v>1640</v>
+      </c>
+      <c r="E97" s="1"/>
       <c r="F97" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G97" s="1"/>
       <c r="H97" s="1" t="s">
@@ -6522,12 +6454,12 @@
       <c r="C98" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="D98" s="11"/>
-      <c r="E98" s="1">
-        <v>872.5</v>
-      </c>
+      <c r="D98" s="11">
+        <v>1745</v>
+      </c>
+      <c r="E98" s="1"/>
       <c r="F98" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" s="1" t="s">
@@ -6561,12 +6493,12 @@
       <c r="C99" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="D99" s="11"/>
-      <c r="E99" s="1">
-        <v>711.5</v>
-      </c>
+      <c r="D99" s="11">
+        <v>1423</v>
+      </c>
+      <c r="E99" s="1"/>
       <c r="F99" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G99" s="1"/>
       <c r="H99" s="1" t="s">
@@ -6600,12 +6532,12 @@
       <c r="C100" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="D100" s="11"/>
-      <c r="E100" s="1">
-        <v>578.5</v>
-      </c>
+      <c r="D100" s="11">
+        <v>1157</v>
+      </c>
+      <c r="E100" s="1"/>
       <c r="F100" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G100" s="1"/>
       <c r="H100" s="1" t="s">
@@ -6639,10 +6571,10 @@
       <c r="C101" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="D101" s="11"/>
-      <c r="E101" s="1">
-        <v>819.69999999999993</v>
-      </c>
+      <c r="D101" s="11">
+        <v>1289</v>
+      </c>
+      <c r="E101" s="1"/>
       <c r="F101" s="1">
         <v>0.3</v>
       </c>
@@ -6678,10 +6610,10 @@
       <c r="C102" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="D102" s="11"/>
-      <c r="E102" s="1">
-        <v>2244.1999999999998</v>
-      </c>
+      <c r="D102" s="11">
+        <v>3206</v>
+      </c>
+      <c r="E102" s="1"/>
       <c r="F102" s="1">
         <v>0.3</v>
       </c>
@@ -6717,10 +6649,10 @@
       <c r="C103" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="D103" s="11"/>
-      <c r="E103" s="1">
-        <v>2939.2</v>
-      </c>
+      <c r="D103" s="11">
+        <v>7348</v>
+      </c>
+      <c r="E103" s="1"/>
       <c r="F103" s="1">
         <v>0.6</v>
       </c>
@@ -6756,10 +6688,10 @@
       <c r="C104" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="D104" s="11"/>
-      <c r="E104" s="1">
-        <v>3423</v>
-      </c>
+      <c r="D104" s="11">
+        <v>4890</v>
+      </c>
+      <c r="E104" s="1"/>
       <c r="F104" s="1">
         <v>0.3</v>
       </c>
@@ -6795,10 +6727,10 @@
       <c r="C105" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="D105" s="11"/>
-      <c r="E105" s="1">
-        <v>3671.5</v>
-      </c>
+      <c r="D105" s="11">
+        <v>5245</v>
+      </c>
+      <c r="E105" s="1"/>
       <c r="F105" s="1">
         <v>0.3</v>
       </c>
@@ -6834,10 +6766,10 @@
       <c r="C106" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="D106" s="11"/>
-      <c r="E106" s="1">
-        <v>2590</v>
-      </c>
+      <c r="D106" s="11">
+        <v>3700</v>
+      </c>
+      <c r="E106" s="1"/>
       <c r="F106" s="1">
         <v>0.3</v>
       </c>
@@ -6873,10 +6805,10 @@
       <c r="C107" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D107" s="11"/>
-      <c r="E107" s="1">
-        <v>1160</v>
-      </c>
+      <c r="D107" s="11">
+        <v>2900</v>
+      </c>
+      <c r="E107" s="1"/>
       <c r="F107" s="1">
         <v>0.6</v>
       </c>
@@ -6912,12 +6844,12 @@
       <c r="C108" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="D108" s="11"/>
-      <c r="E108" s="1">
-        <v>562.5</v>
-      </c>
+      <c r="D108" s="11">
+        <v>1125</v>
+      </c>
+      <c r="E108" s="1"/>
       <c r="F108" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G108" s="1"/>
       <c r="H108" s="1" t="s">
@@ -6951,12 +6883,12 @@
       <c r="C109" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="D109" s="11"/>
-      <c r="E109" s="1">
-        <v>68.599999999999994</v>
-      </c>
+      <c r="D109" s="11">
+        <v>98</v>
+      </c>
+      <c r="E109" s="1"/>
       <c r="F109" s="1">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G109" s="1"/>
       <c r="H109" s="1" t="s">
@@ -6990,10 +6922,10 @@
       <c r="C110" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="D110" s="11"/>
-      <c r="E110" s="1">
-        <v>298.8</v>
-      </c>
+      <c r="D110" s="11">
+        <v>498</v>
+      </c>
+      <c r="E110" s="1"/>
       <c r="F110" s="1">
         <v>0.4</v>
       </c>
@@ -7029,10 +6961,10 @@
       <c r="C111" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="D111" s="11"/>
-      <c r="E111" s="1">
-        <v>348.6</v>
-      </c>
+      <c r="D111" s="11">
+        <v>498</v>
+      </c>
+      <c r="E111" s="1"/>
       <c r="F111" s="1">
         <v>0.3</v>
       </c>
@@ -7068,12 +7000,12 @@
       <c r="C112" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="D112" s="11"/>
-      <c r="E112" s="1">
-        <v>187.5</v>
-      </c>
+      <c r="D112" s="11">
+        <v>395</v>
+      </c>
+      <c r="E112" s="1"/>
       <c r="F112" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G112" s="1"/>
       <c r="H112" s="1" t="s">
@@ -7107,10 +7039,10 @@
       <c r="C113" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="D113" s="11"/>
-      <c r="E113" s="1">
-        <v>688.19999999999993</v>
-      </c>
+      <c r="D113" s="11">
+        <v>1147</v>
+      </c>
+      <c r="E113" s="1"/>
       <c r="F113" s="1">
         <v>0.4</v>
       </c>
@@ -7146,10 +7078,10 @@
       <c r="C114" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="D114" s="11"/>
-      <c r="E114" s="1">
-        <v>613.19999999999993</v>
-      </c>
+      <c r="D114" s="11">
+        <v>1022</v>
+      </c>
+      <c r="E114" s="1"/>
       <c r="F114" s="1">
         <v>0.4</v>
       </c>
@@ -7185,10 +7117,10 @@
       <c r="C115" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="D115" s="11"/>
-      <c r="E115" s="1">
-        <v>561</v>
-      </c>
+      <c r="D115" s="11">
+        <v>1122</v>
+      </c>
+      <c r="E115" s="1"/>
       <c r="F115" s="1">
         <v>0.5</v>
       </c>
@@ -7224,10 +7156,10 @@
       <c r="C116" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="D116" s="11"/>
-      <c r="E116" s="1">
-        <v>1253</v>
-      </c>
+      <c r="D116" s="11">
+        <v>1790</v>
+      </c>
+      <c r="E116" s="1"/>
       <c r="F116" s="1">
         <v>0.3</v>
       </c>
@@ -7263,10 +7195,10 @@
       <c r="C117" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="D117" s="11"/>
-      <c r="E117" s="1">
-        <v>1253</v>
-      </c>
+      <c r="D117" s="11">
+        <v>1790</v>
+      </c>
+      <c r="E117" s="1"/>
       <c r="F117" s="1">
         <v>0.3</v>
       </c>
@@ -7302,10 +7234,10 @@
       <c r="C118" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="D118" s="11"/>
-      <c r="E118" s="1">
-        <v>1253</v>
-      </c>
+      <c r="D118" s="11">
+        <v>1790</v>
+      </c>
+      <c r="E118" s="1"/>
       <c r="F118" s="1">
         <v>0.3</v>
       </c>
@@ -7341,10 +7273,10 @@
       <c r="C119" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="D119" s="11"/>
-      <c r="E119" s="1">
-        <v>284.89999999999998</v>
-      </c>
+      <c r="D119" s="11">
+        <v>407</v>
+      </c>
+      <c r="E119" s="1"/>
       <c r="F119" s="1">
         <v>0.3</v>
       </c>
@@ -7380,10 +7312,10 @@
       <c r="C120" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="D120" s="11"/>
-      <c r="E120" s="1">
-        <v>284.89999999999998</v>
-      </c>
+      <c r="D120" s="11">
+        <v>407</v>
+      </c>
+      <c r="E120" s="1"/>
       <c r="F120" s="1">
         <v>0.3</v>
       </c>
@@ -7419,10 +7351,10 @@
       <c r="C121" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="D121" s="11"/>
-      <c r="E121" s="1">
-        <v>880.8</v>
-      </c>
+      <c r="D121" s="11">
+        <v>1468</v>
+      </c>
+      <c r="E121" s="1"/>
       <c r="F121" s="1">
         <v>0.4</v>
       </c>
@@ -7458,10 +7390,10 @@
       <c r="C122" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="D122" s="11"/>
-      <c r="E122" s="1">
-        <v>1438</v>
-      </c>
+      <c r="D122" s="11">
+        <v>3595</v>
+      </c>
+      <c r="E122" s="1"/>
       <c r="F122" s="1">
         <v>0.6</v>
       </c>
@@ -7497,10 +7429,10 @@
       <c r="C123" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="D123" s="11"/>
-      <c r="E123" s="1">
-        <v>520</v>
-      </c>
+      <c r="D123" s="11">
+        <v>1300</v>
+      </c>
+      <c r="E123" s="1"/>
       <c r="F123" s="1">
         <v>0.6</v>
       </c>
@@ -7536,10 +7468,10 @@
       <c r="C124" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="D124" s="11"/>
-      <c r="E124" s="1">
-        <v>1192</v>
-      </c>
+      <c r="D124" s="11">
+        <v>2980</v>
+      </c>
+      <c r="E124" s="1"/>
       <c r="F124" s="1">
         <v>0.6</v>
       </c>
@@ -7575,10 +7507,10 @@
       <c r="C125" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="D125" s="11"/>
-      <c r="E125" s="1">
-        <v>3390</v>
-      </c>
+      <c r="D125" s="11">
+        <v>6780</v>
+      </c>
+      <c r="E125" s="1"/>
       <c r="F125" s="1">
         <v>0.5</v>
       </c>
@@ -7614,10 +7546,10 @@
       <c r="C126" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="D126" s="11"/>
-      <c r="E126" s="1">
-        <v>1750</v>
-      </c>
+      <c r="D126" s="11">
+        <v>3500</v>
+      </c>
+      <c r="E126" s="1"/>
       <c r="F126" s="1">
         <v>0.5</v>
       </c>
@@ -7653,10 +7585,10 @@
       <c r="C127" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="D127" s="11"/>
-      <c r="E127" s="1">
-        <v>1992</v>
-      </c>
+      <c r="D127" s="11">
+        <v>4980</v>
+      </c>
+      <c r="E127" s="1"/>
       <c r="F127" s="1">
         <v>0.6</v>
       </c>
@@ -7692,10 +7624,10 @@
       <c r="C128" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="D128" s="11"/>
-      <c r="E128" s="1">
-        <v>1992</v>
-      </c>
+      <c r="D128" s="11">
+        <v>4980</v>
+      </c>
+      <c r="E128" s="1"/>
       <c r="F128" s="1">
         <v>0.6</v>
       </c>
@@ -7731,10 +7663,10 @@
       <c r="C129" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D129" s="11"/>
-      <c r="E129" s="1">
-        <v>2880</v>
-      </c>
+      <c r="D129" s="11">
+        <v>5860</v>
+      </c>
+      <c r="E129" s="1"/>
       <c r="F129" s="1">
         <v>0.5</v>
       </c>
@@ -7770,10 +7702,10 @@
       <c r="C130" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="D130" s="11"/>
-      <c r="E130" s="1">
-        <v>2300.9</v>
-      </c>
+      <c r="D130" s="11">
+        <v>3287</v>
+      </c>
+      <c r="E130" s="1"/>
       <c r="F130" s="1">
         <v>0.3</v>
       </c>
@@ -7812,9 +7744,7 @@
       <c r="D131" s="11">
         <v>3640</v>
       </c>
-      <c r="E131" s="1">
-        <v>3640</v>
-      </c>
+      <c r="E131" s="1"/>
       <c r="F131" s="1">
         <v>0.2</v>
       </c>
@@ -7853,9 +7783,7 @@
       <c r="D132" s="12">
         <v>1055</v>
       </c>
-      <c r="E132" s="1">
-        <v>1055</v>
-      </c>
+      <c r="E132" s="1"/>
       <c r="F132" s="1">
         <v>0.2</v>
       </c>
@@ -7892,9 +7820,7 @@
       <c r="D133" s="12">
         <v>3852</v>
       </c>
-      <c r="E133" s="1">
-        <v>3852</v>
-      </c>
+      <c r="E133" s="1"/>
       <c r="F133" s="1">
         <v>0.2</v>
       </c>
@@ -7931,9 +7857,7 @@
       <c r="D134" s="12">
         <v>4332</v>
       </c>
-      <c r="E134" s="1">
-        <v>4332</v>
-      </c>
+      <c r="E134" s="1"/>
       <c r="F134" s="1">
         <v>0.2</v>
       </c>
@@ -7972,9 +7896,7 @@
       <c r="D135" s="12">
         <v>6247</v>
       </c>
-      <c r="E135" s="1">
-        <v>6247</v>
-      </c>
+      <c r="E135" s="1"/>
       <c r="F135" s="1">
         <v>0.2</v>
       </c>
@@ -8013,9 +7935,7 @@
       <c r="D136" s="12">
         <v>1185</v>
       </c>
-      <c r="E136" s="1">
-        <v>1185</v>
-      </c>
+      <c r="E136" s="1"/>
       <c r="F136" s="1">
         <v>0.2</v>
       </c>
@@ -8052,9 +7972,7 @@
       <c r="D137" s="12">
         <v>1089</v>
       </c>
-      <c r="E137" s="1">
-        <v>1089</v>
-      </c>
+      <c r="E137" s="1"/>
       <c r="F137" s="1">
         <v>0.2</v>
       </c>
@@ -8091,9 +8009,7 @@
       <c r="D138" s="12">
         <v>2918</v>
       </c>
-      <c r="E138" s="1">
-        <v>2918</v>
-      </c>
+      <c r="E138" s="1"/>
       <c r="F138" s="1">
         <v>0.2</v>
       </c>
@@ -8130,9 +8046,7 @@
       <c r="D139" s="12">
         <v>2680</v>
       </c>
-      <c r="E139" s="1">
-        <v>2680</v>
-      </c>
+      <c r="E139" s="1"/>
       <c r="F139" s="1">
         <v>0.3</v>
       </c>
@@ -8169,9 +8083,7 @@
       <c r="D140" s="12">
         <v>3192</v>
       </c>
-      <c r="E140" s="1">
-        <v>3192</v>
-      </c>
+      <c r="E140" s="1"/>
       <c r="F140" s="1">
         <v>0.2</v>
       </c>
@@ -8208,9 +8120,7 @@
       <c r="D141" s="12">
         <v>4972</v>
       </c>
-      <c r="E141" s="1">
-        <v>4972</v>
-      </c>
+      <c r="E141" s="1"/>
       <c r="F141" s="1">
         <v>0.2</v>
       </c>
@@ -8247,9 +8157,7 @@
       <c r="D142" s="12">
         <v>9849</v>
       </c>
-      <c r="E142" s="1">
-        <v>9849</v>
-      </c>
+      <c r="E142" s="1"/>
       <c r="F142" s="1">
         <v>0.2</v>
       </c>
@@ -8286,9 +8194,7 @@
       <c r="D143" s="12">
         <v>16233</v>
       </c>
-      <c r="E143" s="1">
-        <v>16233</v>
-      </c>
+      <c r="E143" s="1"/>
       <c r="F143" s="1">
         <v>0.2</v>
       </c>
@@ -8325,9 +8231,7 @@
       <c r="D144" s="12">
         <v>3640</v>
       </c>
-      <c r="E144" s="1">
-        <v>3640</v>
-      </c>
+      <c r="E144" s="1"/>
       <c r="F144" s="1">
         <v>0.2</v>
       </c>
@@ -8710,9 +8614,7 @@
       <c r="D159" s="11">
         <v>6997</v>
       </c>
-      <c r="E159" s="1">
-        <v>6997</v>
-      </c>
+      <c r="E159" s="1"/>
       <c r="F159" s="1">
         <v>0.2</v>
       </c>
@@ -8997,9 +8899,7 @@
       <c r="D170" s="11">
         <v>7756</v>
       </c>
-      <c r="E170" s="1">
-        <v>7756</v>
-      </c>
+      <c r="E170" s="1"/>
       <c r="F170" s="1">
         <v>0.2</v>
       </c>
@@ -9284,9 +9184,7 @@
       <c r="D181" s="12">
         <v>3086</v>
       </c>
-      <c r="E181" s="1">
-        <v>3086</v>
-      </c>
+      <c r="E181" s="1"/>
       <c r="F181" s="1">
         <v>0.2</v>
       </c>
@@ -9321,9 +9219,7 @@
       <c r="D182" s="12">
         <v>4020</v>
       </c>
-      <c r="E182" s="1">
-        <v>4020</v>
-      </c>
+      <c r="E182" s="1"/>
       <c r="F182" s="1">
         <v>0.2</v>
       </c>
@@ -9358,9 +9254,7 @@
       <c r="D183" s="12">
         <v>4605</v>
       </c>
-      <c r="E183" s="1">
-        <v>4605</v>
-      </c>
+      <c r="E183" s="1"/>
       <c r="F183" s="1">
         <v>0.2</v>
       </c>
@@ -9395,9 +9289,7 @@
       <c r="D184" s="12">
         <v>734</v>
       </c>
-      <c r="E184" s="1">
-        <v>734</v>
-      </c>
+      <c r="E184" s="1"/>
       <c r="F184" s="1">
         <v>0.2</v>
       </c>
@@ -9432,9 +9324,7 @@
       <c r="D185" s="12">
         <v>5311</v>
       </c>
-      <c r="E185" s="1">
-        <v>5311</v>
-      </c>
+      <c r="E185" s="1"/>
       <c r="F185" s="1">
         <v>0.2</v>
       </c>
@@ -9669,9 +9559,7 @@
       <c r="D194" s="11">
         <v>3213</v>
       </c>
-      <c r="E194" s="1">
-        <v>3213</v>
-      </c>
+      <c r="E194" s="1"/>
       <c r="F194" s="1">
         <v>0.2</v>
       </c>

</xml_diff>